<commit_message>
Daily slate 2026-06-21 [auto]
</commit_message>
<xml_diff>
--- a/ui_runner/templates/graded_analysis_tabs_2026-06-19.xlsx
+++ b/ui_runner/templates/graded_analysis_tabs_2026-06-19.xlsx
@@ -471,16 +471,16 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>209</v>
+        <v>213</v>
       </c>
       <c r="E2" t="n">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="F2" t="n">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="G2" t="n">
-        <v>46.4</v>
+        <v>46.5</v>
       </c>
     </row>
     <row r="3">
@@ -529,16 +529,16 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>446</v>
+        <v>453</v>
       </c>
       <c r="E4" t="n">
         <v>169</v>
       </c>
       <c r="F4" t="n">
-        <v>277</v>
+        <v>284</v>
       </c>
       <c r="G4" t="n">
-        <v>37.9</v>
+        <v>37.3</v>
       </c>
     </row>
     <row r="5">
@@ -616,16 +616,16 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>106</v>
+        <v>111</v>
       </c>
       <c r="E7" t="n">
-        <v>43</v>
+        <v>48</v>
       </c>
       <c r="F7" t="n">
         <v>63</v>
       </c>
       <c r="G7" t="n">
-        <v>40.6</v>
+        <v>43.2</v>
       </c>
     </row>
     <row r="8">
@@ -674,16 +674,16 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="E9" t="n">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="F9" t="n">
         <v>50</v>
       </c>
       <c r="G9" t="n">
-        <v>39.8</v>
+        <v>40.5</v>
       </c>
     </row>
     <row r="10">
@@ -703,16 +703,16 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>420</v>
+        <v>422</v>
       </c>
       <c r="E10" t="n">
         <v>188</v>
       </c>
       <c r="F10" t="n">
-        <v>232</v>
+        <v>234</v>
       </c>
       <c r="G10" t="n">
-        <v>44.8</v>
+        <v>44.5</v>
       </c>
     </row>
     <row r="11">
@@ -732,16 +732,16 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>981</v>
+        <v>1031</v>
       </c>
       <c r="E11" t="n">
-        <v>610</v>
+        <v>630</v>
       </c>
       <c r="F11" t="n">
-        <v>371</v>
+        <v>401</v>
       </c>
       <c r="G11" t="n">
-        <v>62.2</v>
+        <v>61.1</v>
       </c>
     </row>
     <row r="12">
@@ -761,16 +761,16 @@
         </is>
       </c>
       <c r="D12" t="n">
-        <v>177</v>
+        <v>180</v>
       </c>
       <c r="E12" t="n">
         <v>131</v>
       </c>
       <c r="F12" t="n">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="G12" t="n">
-        <v>74</v>
+        <v>72.8</v>
       </c>
     </row>
     <row r="13">
@@ -819,16 +819,16 @@
         </is>
       </c>
       <c r="D14" t="n">
-        <v>360</v>
+        <v>372</v>
       </c>
       <c r="E14" t="n">
         <v>115</v>
       </c>
       <c r="F14" t="n">
-        <v>245</v>
+        <v>257</v>
       </c>
       <c r="G14" t="n">
-        <v>31.9</v>
+        <v>30.9</v>
       </c>
     </row>
     <row r="15">
@@ -848,16 +848,16 @@
         </is>
       </c>
       <c r="D15" t="n">
-        <v>450</v>
+        <v>458</v>
       </c>
       <c r="E15" t="n">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="F15" t="n">
-        <v>339</v>
+        <v>346</v>
       </c>
       <c r="G15" t="n">
-        <v>24.7</v>
+        <v>24.5</v>
       </c>
     </row>
     <row r="16">
@@ -877,16 +877,16 @@
         </is>
       </c>
       <c r="D16" t="n">
-        <v>249</v>
+        <v>253</v>
       </c>
       <c r="E16" t="n">
         <v>58</v>
       </c>
       <c r="F16" t="n">
-        <v>191</v>
+        <v>195</v>
       </c>
       <c r="G16" t="n">
-        <v>23.3</v>
+        <v>22.9</v>
       </c>
     </row>
     <row r="17">
@@ -906,16 +906,16 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>5018</v>
+        <v>5218</v>
       </c>
       <c r="E17" t="n">
-        <v>1008</v>
+        <v>1025</v>
       </c>
       <c r="F17" t="n">
-        <v>4010</v>
+        <v>4193</v>
       </c>
       <c r="G17" t="n">
-        <v>20.1</v>
+        <v>19.6</v>
       </c>
     </row>
   </sheetData>
@@ -1136,7 +1136,7 @@
         <v>12</v>
       </c>
       <c r="L2" t="n">
-        <v>37.8</v>
+        <v>40.5</v>
       </c>
       <c r="M2" t="n">
         <v>37</v>
@@ -1154,10 +1154,10 @@
         <v>320</v>
       </c>
       <c r="R2" t="n">
-        <v>52.3</v>
+        <v>55.6</v>
       </c>
       <c r="S2" t="n">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="T2" t="n">
         <v>24</v>
@@ -1579,22 +1579,22 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>44.8</v>
+        <v>44.5</v>
       </c>
       <c r="C7" t="n">
-        <v>420</v>
+        <v>422</v>
       </c>
       <c r="D7" t="n">
-        <v>62.2</v>
+        <v>61.1</v>
       </c>
       <c r="E7" t="n">
-        <v>981</v>
+        <v>1031</v>
       </c>
       <c r="F7" t="n">
-        <v>74</v>
+        <v>72.8</v>
       </c>
       <c r="G7" t="n">
-        <v>177</v>
+        <v>180</v>
       </c>
       <c r="H7" t="n">
         <v>49.3</v>
@@ -1603,40 +1603,40 @@
         <v>146</v>
       </c>
       <c r="J7" t="n">
-        <v>31.9</v>
+        <v>30.9</v>
       </c>
       <c r="K7" t="n">
-        <v>360</v>
+        <v>372</v>
       </c>
       <c r="L7" t="n">
-        <v>24.7</v>
+        <v>24.5</v>
       </c>
       <c r="M7" t="n">
-        <v>450</v>
+        <v>458</v>
       </c>
       <c r="N7" t="n">
-        <v>23.3</v>
+        <v>22.9</v>
       </c>
       <c r="O7" t="n">
-        <v>249</v>
+        <v>253</v>
       </c>
       <c r="P7" t="n">
-        <v>20.1</v>
+        <v>19.6</v>
       </c>
       <c r="Q7" t="n">
-        <v>5018</v>
+        <v>5218</v>
       </c>
       <c r="R7" t="n">
-        <v>46.4</v>
+        <v>46.5</v>
       </c>
       <c r="S7" t="n">
-        <v>209</v>
+        <v>213</v>
       </c>
       <c r="T7" t="n">
-        <v>37.9</v>
+        <v>37.3</v>
       </c>
       <c r="U7" t="n">
-        <v>446</v>
+        <v>453</v>
       </c>
       <c r="V7" t="n">
         <v>14.3</v>
@@ -1663,16 +1663,16 @@
         <v>49</v>
       </c>
       <c r="AD7" t="n">
-        <v>40.6</v>
+        <v>43.2</v>
       </c>
       <c r="AE7" t="n">
-        <v>106</v>
+        <v>111</v>
       </c>
       <c r="AF7" t="n">
-        <v>39.8</v>
+        <v>40.5</v>
       </c>
       <c r="AG7" t="n">
-        <v>83</v>
+        <v>84</v>
       </c>
     </row>
   </sheetData>

</xml_diff>